<commit_message>
feat: improve result comprehension (peer reviewed 1)
</commit_message>
<xml_diff>
--- a/data/simulasi_numerik.xlsx
+++ b/data/simulasi_numerik.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3816,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4040,7 +4040,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4264,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4424,7 +4424,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4552,7 +4552,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4616,7 +4616,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4936,7 +4936,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5320,7 +5320,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5768,7 +5768,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5800,7 +5800,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5832,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5928,7 +5928,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5960,7 +5960,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -5992,7 +5992,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6024,7 +6024,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6088,7 +6088,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6152,7 +6152,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6280,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6344,7 +6344,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6504,7 +6504,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6536,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6568,7 +6568,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6728,7 +6728,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6888,7 +6888,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6920,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -6984,7 +6984,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7080,7 +7080,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7112,7 +7112,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7144,7 +7144,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7208,7 +7208,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7240,7 +7240,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7336,7 +7336,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7368,7 +7368,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7432,7 +7432,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7592,7 +7592,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7624,7 +7624,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7656,7 +7656,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7720,7 +7720,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7848,7 +7848,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7912,7 +7912,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7944,7 +7944,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7976,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8040,7 +8040,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8104,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8200,7 +8200,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8232,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8264,7 +8264,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8296,7 +8296,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8328,7 +8328,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8360,7 +8360,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8456,7 +8456,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8488,7 +8488,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8552,7 +8552,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8616,7 +8616,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8648,7 +8648,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8712,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8744,7 +8744,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8808,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8840,7 +8840,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8872,7 +8872,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8904,7 +8904,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8936,7 +8936,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -8968,7 +8968,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9000,7 +9000,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9032,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9096,7 +9096,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9160,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9192,7 +9192,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9256,7 +9256,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9288,7 +9288,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9320,7 +9320,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9352,7 +9352,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9448,7 +9448,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9480,7 +9480,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9512,7 +9512,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9544,7 +9544,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9576,7 +9576,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9640,7 +9640,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>
@@ -9672,7 +9672,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>TIDAK</t>
+          <t>Tidak</t>
         </is>
       </c>
     </row>

</xml_diff>